<commit_message>
Did the reviewe for assignment 1
</commit_message>
<xml_diff>
--- a/Peer_Review_Group_2_Peter_Schoenung.xlsx
+++ b/Peer_Review_Group_2_Peter_Schoenung.xlsx
@@ -8,9 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Grading sheet" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Explanations" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Peer review briefing" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Grading sheet" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Explanations" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Peer review briefing" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="219">
   <si>
     <t xml:space="preserve">Peer-review grading sheet — Chemical Reaction Engineering III, Ulm University</t>
   </si>
@@ -129,24 +129,72 @@
     <t xml:space="preserve">Text quality (language, style, grammar)</t>
   </si>
   <si>
+    <t xml:space="preserve">Nicely readable english. Short enough to be read easily, long enough to get information across in a nice style</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
     <t xml:space="preserve">I-2</t>
   </si>
   <si>
     <t xml:space="preserve">Figures (labels, legends, readability, referenced in text)</t>
   </si>
   <si>
+    <t xml:space="preserve">Good font choice, Style in ICIW style also is a nice choice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legens are way too big to be fit inside the diagrams. More than once there is data beeing obstructed by the legend</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Use matplotlib functionality to clip the legend to the border of the figure, </t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">outside </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">the diagram. Also shorter labels.</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">I-3</t>
   </si>
   <si>
     <t xml:space="preserve">Equations (formatting, variables defined, consistent units)</t>
   </si>
   <si>
+    <t xml:space="preserve">Nicely formatted, indices where needed.</t>
+  </si>
+  <si>
     <t xml:space="preserve">I-4</t>
   </si>
   <si>
     <t xml:space="preserve">Report structure (logical flow, balanced sections, headings)</t>
   </si>
   <si>
+    <t xml:space="preserve">Well structured flow, nice to read.</t>
+  </si>
+  <si>
     <t xml:space="preserve">II) Background &amp; Motivation   (category weight: 20%)</t>
   </si>
   <si>
@@ -156,36 +204,85 @@
     <t xml:space="preserve">Theoretical background (relevant, accurate, linked to assignment)</t>
   </si>
   <si>
+    <t xml:space="preserve">Explanation of how to get to a reaction hypothesis is there, so not 0 points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explanation of the functions used in the code is completely missing. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theoretical Background for the in Code used formulas is a must include. So put it in next time :)</t>
+  </si>
+  <si>
     <t xml:space="preserve">II-2</t>
   </si>
   <si>
     <t xml:space="preserve">Motivation &amp; relevance (why the task matters in reaction engineering)</t>
   </si>
   <si>
+    <t xml:space="preserve">Introduction is well written, theoretical use for exercise is nicely presented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None+</t>
+  </si>
+  <si>
     <t xml:space="preserve">III-1</t>
   </si>
   <si>
     <t xml:space="preserve">FAIR / readable code (comments, variable names, units, structure)</t>
   </si>
   <si>
+    <t xml:space="preserve">Nice commenting for the most part</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explanations of the code cells a bit too generic. Commenting not fully done, e.g. the second residual function has a weighting, which is never explained.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do the code commenting for all the functions and in more detail.</t>
+  </si>
+  <si>
     <t xml:space="preserve">III-2</t>
   </si>
   <si>
     <t xml:space="preserve">Code is supported by report text (methods in code match those described)</t>
   </si>
   <si>
+    <t xml:space="preserve">functions nicely explained outside of the code cells</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a bit short, but that is preferance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explanations outside of the cells in more depht would be nice</t>
+  </si>
+  <si>
     <t xml:space="preserve">III-3</t>
   </si>
   <si>
     <t xml:space="preserve">Documentation of applied methods (reproducible: versions, data, seeds)</t>
   </si>
   <si>
+    <t xml:space="preserve">Everything to full satisfaction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Version of used Python packages would be a nice bonus, but not explicitly needed i think</t>
+  </si>
+  <si>
     <t xml:space="preserve">III-4</t>
   </si>
   <si>
     <t xml:space="preserve">Validation strategy (analytical limits, literature, convergence, sanity checks)</t>
   </si>
   <si>
+    <t xml:space="preserve">A second iteration of the Test is a good start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The second Test is too short, only one parameter is changed. Also the residual Method is not in line with all other reeval methods named with the _ro suffix. This means you are rewriting your eval function. This is even worse because of the jupyter notebook, if you run an above code cell after the reeval one, you are possibly using the wrong function.
+Also, there needs to be another validation tool than just the eye test discussed. Some error statistic like the chi_squared from lmfit itself or the R^2 are possible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reeval needs to be more intensive, a second iteration with now varied reaction orders would have been nice, or a different starting guess for k to see if the solver gets to the same result. </t>
+  </si>
+  <si>
     <t xml:space="preserve">IV) Scientific discussion   (category weight: 35%)</t>
   </si>
   <si>
@@ -195,30 +292,89 @@
     <t xml:space="preserve">Plausibility check of results (orders of magnitude, limiting cases)</t>
   </si>
   <si>
+    <t xml:space="preserve">You checked the k values for plausibility to the reaction speeds observed in the experiments, which is a good point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You say the second fit is better, but that is simply not proven. It even looks like thge fit is worse, at least according to the fit statistics returned by lmfit. There, the chi_squared parameter, wich is a statistical error check, is way bigger for the second iteration. This indicates a  much worse fit, not a better one, like you are saying in the dicussion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement statistical error checks instead of just the ‚it looks good‘ approach. Also discuss more factors and more diverse</t>
+  </si>
+  <si>
     <t xml:space="preserve">IV-2</t>
   </si>
   <si>
     <t xml:space="preserve">Connection to theory (results discussed against background)</t>
   </si>
   <si>
+    <t xml:space="preserve">Discussed the fitted k values against fitting criteria</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Theory missing, discussion against theory therefor mostly also missing.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">One point deduction for too little discussion on the background that is there.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement theory and reflect your results on it.</t>
+  </si>
+  <si>
     <t xml:space="preserve">IV-3</t>
   </si>
   <si>
     <t xml:space="preserve">Significance of the parameter study (informative variation, conclusions drawn)</t>
   </si>
   <si>
+    <t xml:space="preserve">Good fit, k values and model seem to fit and are reasoned that way well enough</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing parameter variation and validation methods still draw into this point. With way to little discussion, the  gained results are too shaky in my opinion. Therefor the conclusions are also too shaky. Also, the just accepting of the second fitting as the beter result without proofing or validating it, is a big miss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do more parameter variation, different approaches, then discuss them in more depht.</t>
+  </si>
+  <si>
     <t xml:space="preserve">IV-4</t>
   </si>
   <si>
     <t xml:space="preserve">Independent interpretation (own reasoning visible, not template-like)</t>
   </si>
   <si>
+    <t xml:space="preserve">Non template formulation in my opinion. Conclusions are self reasoned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conclusion is too short</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discuss more and in more depht. Do that for the missing plausibility checks also, but i dont think a point deduction for that missing is fair here.</t>
+  </si>
+  <si>
     <t xml:space="preserve">IV-5</t>
   </si>
   <si>
     <t xml:space="preserve">Link to industrial application (concrete, realistic scenario)</t>
   </si>
   <si>
+    <t xml:space="preserve">Missing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement it next time :/</t>
+  </si>
+  <si>
     <t xml:space="preserve">V) Critical &amp; transparent AI use   (category weight: 10%)</t>
   </si>
   <si>
@@ -228,6 +384,9 @@
     <t xml:space="preserve">AI transparency (tools, purposes and example prompts clearly documented)</t>
   </si>
   <si>
+    <t xml:space="preserve">All as expected</t>
+  </si>
+  <si>
     <t xml:space="preserve">V-2</t>
   </si>
   <si>
@@ -258,16 +417,101 @@
     <t xml:space="preserve">What the authors should keep doing in future assignments.</t>
   </si>
   <si>
+    <t xml:space="preserve">Your written Text is very nice and readable, formatting is also on point. Kepp going :)
+Code is robust, coding style and variable handling are good (except the hickup with the function, but granted :) )
+Introduction and sources for that are very nice, defenetly expand on that on a theoretical background next time.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Top 3 things to improve</t>
   </si>
   <si>
     <t xml:space="preserve">Concrete, actionable suggestions — refer to the criteria above.</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Do more parameter variation if asked, definetly be more thorough in your code validation
+Discuss your results in more depht than just saying „yeah its good“. Show some objective metric and discuss on it.
+Do </t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">not</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> handle the data like you did here. Just assuming the starting concentrations as 1 and 0 is a sin (even tho you are maybe right, you cant know that!). Setting all data you </t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">assume</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> to be inert to 0 is just very very wrong. If you need to do that, do it on a copy of the data and compare the modified data to the real data. But </t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">never ever ever</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> just modify original data so it fits your theory!</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">One question this report raised for you as a reviewer</t>
   </si>
   <si>
     <t xml:space="preserve">What did reviewing this report make you reflect on for your own work?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data handling is important, setting negative values to 0 is a good idea (because they are physically impossible). Rest of the data handling is kind of a „How not to“ for me :/</t>
   </si>
   <si>
     <t xml:space="preserve">Reminder: Do NOT use AI tools to generate this peer review. Reflecting on someone else's report is the central learning goal of this exercise.</t>
@@ -569,10 +813,10 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0\%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -653,11 +897,26 @@
       <charset val="1"/>
     </font>
     <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -787,7 +1046,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -876,15 +1135,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -896,11 +1159,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -912,7 +1175,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -996,193 +1259,18 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1f497d"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="eeece1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4f81bd"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="c0504d"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9bbb59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064a2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4bacc6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="f79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ff"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H58"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="37.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="10.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="32"/>
   </cols>
   <sheetData>
@@ -1417,17 +1505,25 @@
       <c r="D19" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
+      <c r="E19" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C20" s="21" t="n">
         <v>0.1</v>
@@ -1435,17 +1531,25 @@
       <c r="D20" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
+      <c r="E20" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="H20" s="18" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C21" s="16" t="n">
         <v>0.1</v>
@@ -1453,17 +1557,25 @@
       <c r="D21" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
+      <c r="E21" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H21" s="18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C22" s="21" t="n">
         <v>0.1</v>
@@ -1471,14 +1583,22 @@
       <c r="D22" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="E22" s="17"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
+      <c r="E22" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H22" s="18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
@@ -1490,10 +1610,10 @@
     </row>
     <row r="24" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C24" s="16" t="n">
         <v>0.2</v>
@@ -1501,17 +1621,25 @@
       <c r="D24" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="E24" s="17"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
+      <c r="E24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="H24" s="18" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C25" s="21" t="n">
         <v>0.2</v>
@@ -1519,10 +1647,18 @@
       <c r="D25" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="E25" s="17"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
+      <c r="E25" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G25" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="18" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14"/>
@@ -1534,12 +1670,12 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
     </row>
-    <row r="27" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C27" s="16" t="n">
         <v>0.25</v>
@@ -1547,17 +1683,25 @@
       <c r="D27" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="E27" s="17"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
+      <c r="E27" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="H27" s="18" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="C28" s="21" t="n">
         <v>0.25</v>
@@ -1565,17 +1709,25 @@
       <c r="D28" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="E28" s="17"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
+      <c r="E28" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="H28" s="22" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C29" s="16" t="n">
         <v>0.25</v>
@@ -1583,17 +1735,25 @@
       <c r="D29" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="E29" s="17"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="18"/>
-    </row>
-    <row r="30" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E29" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H29" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="186" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="C30" s="21" t="n">
         <v>0.25</v>
@@ -1601,14 +1761,22 @@
       <c r="D30" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="E30" s="17"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
+      <c r="E30" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H30" s="18" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
@@ -1618,12 +1786,12 @@
       <c r="G31" s="14"/>
       <c r="H31" s="14"/>
     </row>
-    <row r="32" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="120.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="C32" s="16" t="n">
         <v>0.35</v>
@@ -1631,17 +1799,25 @@
       <c r="D32" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="E32" s="17"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-    </row>
-    <row r="33" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E32" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="G32" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="H32" s="18" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="C33" s="21" t="n">
         <v>0.35</v>
@@ -1649,17 +1825,25 @@
       <c r="D33" s="21" t="n">
         <v>0.2</v>
       </c>
-      <c r="E33" s="17"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-    </row>
-    <row r="34" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E33" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="H33" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="106.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="C34" s="16" t="n">
         <v>0.35</v>
@@ -1667,17 +1851,25 @@
       <c r="D34" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="E34" s="17"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
-    </row>
-    <row r="35" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E34" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="H34" s="18" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="59.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="C35" s="21" t="n">
         <v>0.35</v>
@@ -1685,17 +1877,25 @@
       <c r="D35" s="21" t="n">
         <v>0.2</v>
       </c>
-      <c r="E35" s="17"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
+      <c r="E35" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="H35" s="18" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>64</v>
+        <v>99</v>
       </c>
       <c r="C36" s="16" t="n">
         <v>0.35</v>
@@ -1703,29 +1903,35 @@
       <c r="D36" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="E36" s="17"/>
+      <c r="E36" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
+      <c r="G36" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="H36" s="18" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
+      <c r="A37" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C38" s="16" t="n">
         <v>0.1</v>
@@ -1733,17 +1939,25 @@
       <c r="D38" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="E38" s="17"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
+      <c r="E38" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H38" s="18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>69</v>
+        <v>107</v>
       </c>
       <c r="C39" s="21" t="n">
         <v>0.1</v>
@@ -1751,14 +1965,22 @@
       <c r="D39" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="E39" s="17"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
+      <c r="E39" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G39" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H39" s="18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -1770,41 +1992,41 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>71</v>
+        <v>109</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
-      <c r="E42" s="23" t="n">
+      <c r="E42" s="24" t="n">
         <f aca="false">((0.025*E19) + (0.025*E20) + (0.025*E21) + (0.025*E22) + (0.1*E24) + (0.1*E25) + (0.0625*E27) + (0.0625*E28) + (0.0625*E29) + (0.0625*E30) + (0.07*E32) + (0.07*E33) + (0.07*E34) + (0.07*E35) + (0.07*E36) + (0.05*E38) + (0.05*E39))/4</f>
-        <v>0</v>
+        <v>0.68125</v>
       </c>
       <c r="F42" s="12" t="s">
-        <v>72</v>
+        <v>110</v>
       </c>
       <c r="G42" s="12"/>
       <c r="H42" s="12"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>73</v>
+        <v>111</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
-      <c r="E43" s="24" t="n">
+      <c r="E43" s="25" t="n">
         <f aca="false">E42*100</f>
-        <v>0</v>
+        <v>68.125</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="G43" s="12"/>
       <c r="H43" s="12"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
@@ -1815,118 +2037,124 @@
       <c r="H45" s="6"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="B46" s="25"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="25"/>
-      <c r="G46" s="25"/>
-      <c r="H46" s="25"/>
+      <c r="A46" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B46" s="26"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="26"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B47" s="26"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="26"/>
+      <c r="A47" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="B47" s="27"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
     </row>
     <row r="48" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="27"/>
-      <c r="B48" s="27"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="27"/>
-      <c r="E48" s="27"/>
-      <c r="F48" s="27"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
+      <c r="A48" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="B48" s="28"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="28"/>
+      <c r="G48" s="28"/>
+      <c r="H48" s="28"/>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="B50" s="25"/>
-      <c r="C50" s="25"/>
-      <c r="D50" s="25"/>
-      <c r="E50" s="25"/>
-      <c r="F50" s="25"/>
-      <c r="G50" s="25"/>
-      <c r="H50" s="25"/>
+      <c r="A50" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="B50" s="26"/>
+      <c r="C50" s="26"/>
+      <c r="D50" s="26"/>
+      <c r="E50" s="26"/>
+      <c r="F50" s="26"/>
+      <c r="G50" s="26"/>
+      <c r="H50" s="26"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="B51" s="26"/>
-      <c r="C51" s="26"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="26"/>
-      <c r="F51" s="26"/>
-      <c r="G51" s="26"/>
-      <c r="H51" s="26"/>
+      <c r="A51" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="B51" s="27"/>
+      <c r="C51" s="27"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="27"/>
+      <c r="G51" s="27"/>
+      <c r="H51" s="27"/>
     </row>
     <row r="52" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="27"/>
-      <c r="B52" s="27"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="27"/>
+      <c r="A52" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="B52" s="28"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="28"/>
+      <c r="H52" s="28"/>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B54" s="25"/>
-      <c r="C54" s="25"/>
-      <c r="D54" s="25"/>
-      <c r="E54" s="25"/>
-      <c r="F54" s="25"/>
-      <c r="G54" s="25"/>
-      <c r="H54" s="25"/>
+      <c r="A54" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="B54" s="26"/>
+      <c r="C54" s="26"/>
+      <c r="D54" s="26"/>
+      <c r="E54" s="26"/>
+      <c r="F54" s="26"/>
+      <c r="G54" s="26"/>
+      <c r="H54" s="26"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="B55" s="26"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
-      <c r="G55" s="26"/>
-      <c r="H55" s="26"/>
+      <c r="A55" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="B55" s="27"/>
+      <c r="C55" s="27"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="27"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="27"/>
+      <c r="H55" s="27"/>
     </row>
     <row r="56" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="27"/>
-      <c r="B56" s="27"/>
-      <c r="C56" s="27"/>
-      <c r="D56" s="27"/>
-      <c r="E56" s="27"/>
-      <c r="F56" s="27"/>
-      <c r="G56" s="27"/>
-      <c r="H56" s="27"/>
+      <c r="A56" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="B56" s="28"/>
+      <c r="C56" s="28"/>
+      <c r="D56" s="28"/>
+      <c r="E56" s="28"/>
+      <c r="F56" s="28"/>
+      <c r="G56" s="28"/>
+      <c r="H56" s="28"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="B58" s="28"/>
-      <c r="C58" s="28"/>
-      <c r="D58" s="28"/>
-      <c r="E58" s="28"/>
-      <c r="F58" s="28"/>
-      <c r="G58" s="28"/>
-      <c r="H58" s="28"/>
+      <c r="A58" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="B58" s="29"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
+      <c r="E58" s="29"/>
+      <c r="F58" s="29"/>
+      <c r="G58" s="29"/>
+      <c r="H58" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="39">
@@ -1971,18 +2199,18 @@
     <mergeCell ref="A58:H58"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter a value between 0 and 4 (half points allowed)." errorStyle="stop" errorTitle="Invalid score" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E19:E22 E24:E25 E27:E30 E32:E36 E38:E39" type="decimal">
+    <dataValidation allowBlank="true" error="Please enter a value between 0 and 4 (half points allowed)." errorTitle="Invalid score" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E19:E22 E24:E25 E27:E30 E32:E36 E38:E39" type="decimal">
       <formula1>0</formula1>
       <formula2>4</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1991,21 +2219,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="37.99"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>124</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2020,302 +2248,302 @@
         <v>25</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>84</v>
+        <v>125</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>86</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="D3" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="E3" s="30" t="s">
-        <v>90</v>
+      <c r="B3" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="31" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>94</v>
+        <v>37</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="E5" s="30" t="s">
-        <v>98</v>
+        <v>42</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>100</v>
-      </c>
-      <c r="D6" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="E6" s="30" t="s">
-        <v>102</v>
+        <v>45</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>142</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="D7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="E7" s="30" t="s">
-        <v>106</v>
+        <v>49</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="D8" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="E8" s="30" t="s">
-        <v>110</v>
+        <v>54</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>150</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>111</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="D9" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="E9" s="30" t="s">
-        <v>114</v>
+        <v>58</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="E9" s="31" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>115</v>
-      </c>
-      <c r="C10" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="D10" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="E10" s="30" t="s">
-        <v>118</v>
+        <v>63</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="D11" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="E11" s="30" t="s">
-        <v>122</v>
+        <v>68</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>162</v>
+      </c>
+      <c r="E11" s="31" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>124</v>
-      </c>
-      <c r="D12" s="30" t="s">
-        <v>125</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>126</v>
+        <v>72</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>165</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="D13" s="30" t="s">
-        <v>129</v>
-      </c>
-      <c r="E13" s="30" t="s">
-        <v>130</v>
+        <v>78</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13" s="31" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>132</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="E14" s="30" t="s">
-        <v>134</v>
+        <v>83</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>174</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>135</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="D15" s="30" t="s">
-        <v>137</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>138</v>
+        <v>88</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>176</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>177</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>178</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="C16" s="30" t="s">
-        <v>140</v>
-      </c>
-      <c r="D16" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>142</v>
+        <v>93</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>180</v>
+      </c>
+      <c r="C16" s="31" t="s">
+        <v>181</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>182</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="D17" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>146</v>
+        <v>98</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>186</v>
+      </c>
+      <c r="E17" s="31" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>147</v>
-      </c>
-      <c r="C18" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="E18" s="30" t="s">
-        <v>150</v>
+        <v>103</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="D18" s="32" t="s">
+        <v>190</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>154</v>
+        <v>106</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>193</v>
+      </c>
+      <c r="D19" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2323,8 +2551,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2333,175 +2561,175 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="32" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" s="32"/>
+      <c r="A2" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
       <c r="B3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
-        <v>158</v>
-      </c>
-      <c r="B4" s="32"/>
+      <c r="A4" s="33" t="s">
+        <v>199</v>
+      </c>
+      <c r="B4" s="33"/>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="33" t="s">
-        <v>159</v>
+      <c r="A5" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>160</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="33" t="s">
-        <v>159</v>
+      <c r="A6" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>161</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="33" t="s">
-        <v>159</v>
+      <c r="A7" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>162</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="33" t="s">
-        <v>159</v>
+      <c r="A8" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>163</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="s">
-        <v>159</v>
+      <c r="A9" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>164</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="s">
-        <v>165</v>
-      </c>
-      <c r="B10" s="32"/>
+      <c r="A10" s="33" t="s">
+        <v>206</v>
+      </c>
+      <c r="B10" s="33"/>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="s">
-        <v>159</v>
+      <c r="A11" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>166</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="33" t="s">
-        <v>159</v>
+      <c r="A12" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>167</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="33" t="s">
-        <v>159</v>
+      <c r="A13" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>168</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="32" t="s">
-        <v>169</v>
-      </c>
-      <c r="B14" s="32"/>
+      <c r="A14" s="33" t="s">
+        <v>210</v>
+      </c>
+      <c r="B14" s="33"/>
     </row>
     <row r="15" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>170</v>
+        <v>211</v>
       </c>
       <c r="B15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
-        <v>171</v>
-      </c>
-      <c r="B16" s="32"/>
+      <c r="A16" s="33" t="s">
+        <v>212</v>
+      </c>
+      <c r="B16" s="33"/>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="33" t="s">
-        <v>159</v>
+      <c r="A17" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="33" t="s">
-        <v>159</v>
+      <c r="A18" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>173</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="33" t="s">
-        <v>159</v>
+      <c r="A19" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>174</v>
+        <v>215</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="33" t="s">
-        <v>159</v>
+      <c r="A20" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>175</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="33" t="s">
-        <v>159</v>
+      <c r="A21" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>176</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="33" t="s">
-        <v>159</v>
+      <c r="A22" s="34" t="s">
+        <v>200</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>177</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -2516,8 +2744,8 @@
     <mergeCell ref="A16:B16"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>